<commit_message>
feat: add configurable post-upload validation framework and product price UI validation
- Add ScenarioData sheet support in ExcelLoader
- Pass validateMode and scenarioData to PostUploadValidator
- Refactor PostUploadValidator using validation mode handlers
- Add PROD_PRICE validation flow
- Implement PurchasePricePage and reusable basePage
- Validate generated Excel prices against Purchase Price UI
- Improve Excel numeric value generation for long numbers
- Add validation pass messages to TestSummary
- Update LMT validation to report ValidationResult
- Add configurable Chrome zoom setting
- Refactor UI search validation into a reusable method
</commit_message>
<xml_diff>
--- a/ResourcesBD/configBD.xlsx
+++ b/ResourcesBD/configBD.xlsx
@@ -9,12 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="4100"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="4100" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Screens" sheetId="1" r:id="rId1"/>
-    <sheet name="Params" sheetId="2" r:id="rId2"/>
-    <sheet name="Rules" sheetId="3" r:id="rId3"/>
+    <sheet name="Validations" sheetId="4" r:id="rId1"/>
+    <sheet name="Screens" sheetId="1" r:id="rId2"/>
+    <sheet name="Params" sheetId="2" r:id="rId3"/>
+    <sheet name="Rules" sheetId="3" r:id="rId4"/>
+    <sheet name="ScenarioData" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="196">
   <si>
     <t>screenName</t>
   </si>
@@ -478,14 +480,149 @@
     <t>NIC</t>
   </si>
   <si>
+    <t>validateMode</t>
+  </si>
+  <si>
+    <t>menuSearch</t>
+  </si>
+  <si>
+    <t>validateScreenId</t>
+  </si>
+  <si>
+    <t>validateGeneratedCol</t>
+  </si>
+  <si>
+    <t>columnId</t>
+  </si>
+  <si>
+    <t>UI_Search</t>
+  </si>
+  <si>
+    <t>dsr profile hq</t>
+  </si>
+  <si>
+    <t>DYL_202044</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__EPP2DESC</t>
+  </si>
+  <si>
+    <t>product Enrichment Approval</t>
+  </si>
+  <si>
+    <t>Outlet profile HQ</t>
+  </si>
+  <si>
+    <t>DYL_BG1013</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__EPP1DESC</t>
+  </si>
+  <si>
+    <t>Section Creation HQ</t>
+  </si>
+  <si>
+    <t>DYL_202046</t>
+  </si>
+  <si>
+    <t>Section Code</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__ENTITYCODE</t>
+  </si>
+  <si>
+    <t>Distributor Profile HQ</t>
+  </si>
+  <si>
+    <t>DYL_L__BusinessEntityProfile</t>
+  </si>
+  <si>
+    <t>Distributor Name*</t>
+  </si>
+  <si>
+    <t>Vehicle Profile</t>
+  </si>
+  <si>
+    <t>DYL_1032</t>
+  </si>
+  <si>
+    <t>Description*</t>
+  </si>
+  <si>
+    <t>rowfilter_Description</t>
+  </si>
+  <si>
+    <t>Price Master Approval</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>bulk order upload</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>User profile</t>
+  </si>
+  <si>
+    <t>0201</t>
+  </si>
+  <si>
+    <t>rowfilter_code</t>
+  </si>
+  <si>
+    <t>SECTION</t>
+  </si>
+  <si>
+    <t>AUTOSEC</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>PriceToValidate</t>
+  </si>
+  <si>
+    <t>priceScreenID</t>
+  </si>
+  <si>
+    <t>tradePriceCTN</t>
+  </si>
+  <si>
+    <t>PROD_PRICE</t>
+  </si>
+  <si>
+    <t>ScreenName</t>
+  </si>
+  <si>
+    <t>ScreenId</t>
+  </si>
+  <si>
+    <t>PURCHASE PRICE</t>
+  </si>
+  <si>
+    <t>PURCHASE_PRICE</t>
+  </si>
+  <si>
+    <t>Product Code</t>
+  </si>
+  <si>
+    <t>65150683</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -501,8 +638,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -521,8 +664,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -569,11 +718,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -611,6 +799,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -891,7 +1099,387 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A3" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>159</v>
+      </c>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+    </row>
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="31.54296875" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -900,9 +1488,10 @@
     <col min="4" max="4" width="34.6328125" customWidth="1"/>
     <col min="5" max="5" width="39.08984375" customWidth="1"/>
     <col min="6" max="6" width="10.36328125" customWidth="1"/>
+    <col min="7" max="7" width="13.81640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>98</v>
       </c>
@@ -918,11 +1507,14 @@
       <c r="E1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="28" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" s="6" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G1" s="21" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="6" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>99</v>
       </c>
@@ -938,11 +1530,14 @@
       <c r="E2" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="7" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F2" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="7" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>100</v>
       </c>
@@ -958,11 +1553,12 @@
       <c r="E3" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F3" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G3" s="12"/>
+    </row>
+    <row r="4" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>101</v>
       </c>
@@ -978,11 +1574,14 @@
       <c r="E4" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="29" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" s="6" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G4" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="6" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>103</v>
       </c>
@@ -998,11 +1597,14 @@
       <c r="E5" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F5" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>104</v>
       </c>
@@ -1013,16 +1615,19 @@
         <v>45</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F6" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>105</v>
       </c>
@@ -1033,16 +1638,19 @@
         <v>61</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F7" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>106</v>
       </c>
@@ -1053,16 +1661,17 @@
         <v>65</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F8" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>107</v>
       </c>
@@ -1078,11 +1687,12 @@
       <c r="E9" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F9" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>108</v>
       </c>
@@ -1098,11 +1708,12 @@
       <c r="E10" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F10" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G10" s="12"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>110</v>
       </c>
@@ -1113,16 +1724,19 @@
         <v>112</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="F11" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F11" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>102</v>
       </c>
@@ -1136,11 +1750,12 @@
         <v>43</v>
       </c>
       <c r="E12" s="12"/>
-      <c r="F12" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F12" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>121</v>
       </c>
@@ -1156,11 +1771,12 @@
       <c r="E13" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F13" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G13" s="12"/>
+    </row>
+    <row r="14" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>122</v>
       </c>
@@ -1176,11 +1792,12 @@
       <c r="E14" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="19" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F14" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" s="19" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="18" t="s">
         <v>125</v>
       </c>
@@ -1196,11 +1813,13 @@
       <c r="E15" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="19" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F15" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G15" s="12"/>
+      <c r="H15" s="30"/>
+    </row>
+    <row r="16" spans="1:8" s="19" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="18" t="s">
         <v>129</v>
       </c>
@@ -1216,11 +1835,13 @@
       <c r="E16" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F16" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G16" s="12"/>
+      <c r="H16" s="30"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="18" t="s">
         <v>133</v>
       </c>
@@ -1236,11 +1857,14 @@
       <c r="E17" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="F17" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F17" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="20" t="s">
         <v>137</v>
       </c>
@@ -1256,9 +1880,10 @@
       <c r="E18" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="F18" s="11" t="s">
-        <v>76</v>
-      </c>
+      <c r="F18" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="G18" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1266,7 +1891,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="19" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1372,7 +1997,7 @@
       </c>
       <c r="D7" s="4" t="str">
         <f ca="1" xml:space="preserve"> TEXT(TODAY() - 4, "yyyy-mm-dd")</f>
-        <v>2026-05-04</v>
+        <v>2026-06-25</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1387,7 +2012,7 @@
       </c>
       <c r="D8" s="5" t="str">
         <f ca="1">TEXT(TODAY()+2, "yyyy-mm-dd")</f>
-        <v>2026-05-10</v>
+        <v>2026-07-01</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1676,16 +2301,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="24.36328125" customWidth="1"/>
     <col min="3" max="3" width="22.90625" customWidth="1"/>
     <col min="4" max="4" width="13.7265625" customWidth="1"/>
     <col min="5" max="5" width="6.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
@@ -2014,7 +2639,148 @@
         <v>17</v>
       </c>
     </row>
+    <row r="19" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="2">
+        <v>5</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="2">
+        <v>4</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="2">
+        <v>4</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="13.7265625" customWidth="1"/>
+    <col min="3" max="3" width="15.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(validation): add UI and Excel validation workflows with page objects
- Add Product, Distributor Profile, Company Mapping, and Order Booking page objects
- Implement product enrichment and distributor profile UI validations
- Add uploaded vs downloaded Excel comparison validation
- Add order booking validation message verification
- Refactor PostUploadValidator to support multiple validation modes
- Improve navigation and dropdown handling in basePage
- Use robust click for proceed button and menu navigation
- Append validation results to test summary
- Enhance HTML test summary formatting
- Reorder download/upload flow for DOWNLOAD_UPDATE_UPLOAD
</commit_message>
<xml_diff>
--- a/ResourcesBD/configBD.xlsx
+++ b/ResourcesBD/configBD.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="237">
   <si>
     <t>screenName</t>
   </si>
@@ -246,376 +246,500 @@
     <t>BASE_PACK_EXCEL</t>
   </si>
   <si>
+    <t>ProductEnrichmentComponentApproval.xlsx</t>
+  </si>
+  <si>
+    <t>DOWNLOAD_UPDATE_UPLOAD</t>
+  </si>
+  <si>
+    <t>DOWNLOAD_UPLOAD</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>CNIC Number</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>LUX</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Price Master Excel</t>
+  </si>
+  <si>
+    <t>geoCode</t>
+  </si>
+  <si>
+    <t>Vehicle Master Bulk Upload</t>
+  </si>
+  <si>
+    <t>001001-GT/MT</t>
+  </si>
+  <si>
+    <t>distCode</t>
+  </si>
+  <si>
+    <t>M/S. ATLANTIC DISTRIBUTION</t>
+  </si>
+  <si>
+    <t>LUX SHOWER 220ML BANDED</t>
+  </si>
+  <si>
+    <t>shahmeer OB PJP OTC2</t>
+  </si>
+  <si>
+    <t>Pureit Careline</t>
+  </si>
+  <si>
+    <t>Product Enrichment Excel Upload Approval</t>
+  </si>
+  <si>
+    <t>002001-GT/MT</t>
+  </si>
+  <si>
+    <t>15437620-M/S. ATLANTIC DISTRIBUTION</t>
+  </si>
+  <si>
+    <t>15437620-leopardPOB-leopardPOB</t>
+  </si>
+  <si>
+    <t>Wholesale</t>
+  </si>
+  <si>
+    <t>SKIN CLEANSING</t>
+  </si>
+  <si>
+    <t>LUX SKIN CLEANSING BAR FOREVER 25G</t>
+  </si>
+  <si>
+    <t>LUX BAR FOREVER CP_W_CORE 216X25G</t>
+  </si>
+  <si>
+    <t>testID</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Bulk Order Upload</t>
+  </si>
+  <si>
+    <t>DYL_LMT_ORDER_CREATION</t>
+  </si>
+  <si>
+    <t>LMT</t>
+  </si>
+  <si>
+    <t>LmtOrderCreationExcel.xlsx</t>
+  </si>
+  <si>
+    <t>PO_NUMBER</t>
+  </si>
+  <si>
+    <t>0000000135</t>
+  </si>
+  <si>
+    <t>Product Exclusion Policy</t>
+  </si>
+  <si>
+    <t>PRODUCT_POLICY</t>
+  </si>
+  <si>
+    <t>PEP</t>
+  </si>
+  <si>
+    <t>ProductExclusionFile.xlsx</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>ProductExclusionFile1.xlsx</t>
+  </si>
+  <si>
+    <t>00Access2024-RQBTESTING</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Distributor shuffling upload</t>
+  </si>
+  <si>
+    <t>DISTRIBUTOR_SHUFFLING_UPLOAD</t>
+  </si>
+  <si>
+    <t>DistributorShuffling1.xlsx</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>UPLOAD_ONLY</t>
+  </si>
+  <si>
+    <t>DistributorShuffling2.xlsx</t>
+  </si>
+  <si>
+    <t>Distributor Shuffling Upload</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>User Bulk Upload</t>
+  </si>
+  <si>
+    <t>USER_BULK_UPLOAD</t>
+  </si>
+  <si>
+    <t>UserBulkUpload.xlsx</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Selling Category Bulk Upload</t>
+  </si>
+  <si>
+    <t>SELLING_CATEGORY_BULK_UPLOAD</t>
+  </si>
+  <si>
+    <t>Selling_Category_Bulk_Upload.xlsx</t>
+  </si>
+  <si>
+    <t>leopardPOB - leopardPOB</t>
+  </si>
+  <si>
+    <t>RQBTESTING</t>
+  </si>
+  <si>
+    <t>DEWANHAT</t>
+  </si>
+  <si>
+    <t>DISTRIBUTOR</t>
+  </si>
+  <si>
+    <t>Code*</t>
+  </si>
+  <si>
+    <t>User_</t>
+  </si>
+  <si>
+    <t>Name*</t>
+  </si>
+  <si>
+    <t>Auto_</t>
+  </si>
+  <si>
+    <t>NIC</t>
+  </si>
+  <si>
+    <t>validateMode</t>
+  </si>
+  <si>
+    <t>menuSearch</t>
+  </si>
+  <si>
+    <t>validateScreenId</t>
+  </si>
+  <si>
+    <t>validateGeneratedCol</t>
+  </si>
+  <si>
+    <t>columnId</t>
+  </si>
+  <si>
+    <t>UI_Search</t>
+  </si>
+  <si>
+    <t>dsr profile hq</t>
+  </si>
+  <si>
+    <t>DYL_202044</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__EPP2DESC</t>
+  </si>
+  <si>
+    <t>product Enrichment Approval</t>
+  </si>
+  <si>
+    <t>Outlet profile HQ</t>
+  </si>
+  <si>
+    <t>DYL_BG1013</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__EPP1DESC</t>
+  </si>
+  <si>
+    <t>Section Creation HQ</t>
+  </si>
+  <si>
+    <t>DYL_202046</t>
+  </si>
+  <si>
+    <t>Section Code</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__ENTITYCODE</t>
+  </si>
+  <si>
+    <t>Distributor Profile HQ</t>
+  </si>
+  <si>
+    <t>DYL_L__BusinessEntityProfile</t>
+  </si>
+  <si>
+    <t>Distributor Name*</t>
+  </si>
+  <si>
+    <t>Vehicle Profile</t>
+  </si>
+  <si>
+    <t>DYL_1032</t>
+  </si>
+  <si>
+    <t>Description*</t>
+  </si>
+  <si>
+    <t>rowfilter_Description</t>
+  </si>
+  <si>
+    <t>Price Master Approval</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>bulk order upload</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>User profile</t>
+  </si>
+  <si>
+    <t>0201</t>
+  </si>
+  <si>
+    <t>rowfilter_code</t>
+  </si>
+  <si>
+    <t>SECTION</t>
+  </si>
+  <si>
+    <t>AUTOSEC</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>PriceToValidate</t>
+  </si>
+  <si>
+    <t>priceScreenID</t>
+  </si>
+  <si>
+    <t>tradePriceCTN</t>
+  </si>
+  <si>
+    <t>PROD_PRICE</t>
+  </si>
+  <si>
+    <t>ScreenId</t>
+  </si>
+  <si>
+    <t>PURCHASE PRICE</t>
+  </si>
+  <si>
+    <t>PURCHASE_PRICE</t>
+  </si>
+  <si>
+    <t>Product Code</t>
+  </si>
+  <si>
+    <t>65150683</t>
+  </si>
+  <si>
+    <t>ProductEnrichment.xlsx</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product Enrichment Excel </t>
+  </si>
+  <si>
+    <t>NG1102</t>
+  </si>
+  <si>
+    <t>PROD_ENRICH</t>
+  </si>
+  <si>
+    <t>Product Enrichment</t>
+  </si>
+  <si>
+    <t>Short Description</t>
+  </si>
+  <si>
+    <t>AUTO_PROD</t>
+  </si>
+  <si>
+    <t>68453705</t>
+  </si>
+  <si>
+    <t>FieldToValidate</t>
+  </si>
+  <si>
+    <t>DYL_102003024</t>
+  </si>
+  <si>
+    <t>Product Configuration</t>
+  </si>
+  <si>
+    <t>txt__pprd_abrv</t>
+  </si>
+  <si>
+    <t>attributeScreenID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product Enrichment </t>
+  </si>
+  <si>
+    <t>Spending Time</t>
+  </si>
+  <si>
+    <t>DIST_PROFILE</t>
+  </si>
+  <si>
+    <t>DistCode</t>
+  </si>
+  <si>
+    <t>TXT__EPP1SPENDINGTIME</t>
+  </si>
+  <si>
+    <t>15437620</t>
+  </si>
+  <si>
+    <t>dsrType</t>
+  </si>
+  <si>
+    <t>PJPNO</t>
+  </si>
+  <si>
+    <t>SELLCAT</t>
+  </si>
+  <si>
+    <t>OUTLET</t>
+  </si>
+  <si>
+    <t>Order Booker</t>
+  </si>
+  <si>
+    <t>0000000361-JAGUAR PJP OB</t>
+  </si>
+  <si>
+    <t>Full Range Selling Category</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>C0000023667-Shahjalal Super Store</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>order booking</t>
+  </si>
+  <si>
+    <t>ORDER_BOOKING</t>
+  </si>
+  <si>
+    <t>VALID_EXCEL</t>
+  </si>
+  <si>
+    <t>ExpectedMessage</t>
+  </si>
+  <si>
+    <t>SKU 20099831  Quantity Restricted From 500.00000000 To 50000.00000000</t>
+  </si>
+  <si>
+    <t>QuantityPCS</t>
+  </si>
+  <si>
+    <t>0099831</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>CompareColumns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base Pack, BasePack Description, Lead Base Pack, LeadBasePack Description,status
+</t>
+  </si>
+  <si>
+    <t>COMPARE</t>
+  </si>
+  <si>
     <t>basepack.xlsx</t>
   </si>
   <si>
-    <t>ProductEnrichmentComponentApproval.xlsx</t>
-  </si>
-  <si>
-    <t>DOWNLOAD_UPDATE_UPLOAD</t>
-  </si>
-  <si>
-    <t>DOWNLOAD_UPLOAD</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>CNIC Number</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>LUX</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>Price Master Excel</t>
-  </si>
-  <si>
-    <t>geoCode</t>
-  </si>
-  <si>
-    <t>Vehicle Master Bulk Upload</t>
-  </si>
-  <si>
-    <t>001001-GT/MT</t>
-  </si>
-  <si>
-    <t>distCode</t>
-  </si>
-  <si>
-    <t>M/S. ATLANTIC DISTRIBUTION</t>
-  </si>
-  <si>
-    <t>LUX SHOWER 220ML BANDED</t>
-  </si>
-  <si>
-    <t>shahmeer OB PJP OTC2</t>
-  </si>
-  <si>
-    <t>Pureit Careline</t>
-  </si>
-  <si>
-    <t>Product Enrichment Excel Upload Approval</t>
-  </si>
-  <si>
-    <t>002001-GT/MT</t>
-  </si>
-  <si>
-    <t>15437620-M/S. ATLANTIC DISTRIBUTION</t>
-  </si>
-  <si>
-    <t>15437620-leopardPOB-leopardPOB</t>
-  </si>
-  <si>
-    <t>Wholesale</t>
-  </si>
-  <si>
-    <t>SKIN CLEANSING</t>
-  </si>
-  <si>
-    <t>LUX SKIN CLEANSING BAR FOREVER 25G</t>
-  </si>
-  <si>
-    <t>LUX BAR FOREVER CP_W_CORE 216X25G</t>
-  </si>
-  <si>
-    <t>testID</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>07</t>
-  </si>
-  <si>
-    <t>08</t>
-  </si>
-  <si>
-    <t>09</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>Bulk Order Upload</t>
-  </si>
-  <si>
-    <t>DYL_LMT_ORDER_CREATION</t>
-  </si>
-  <si>
-    <t>LMT</t>
-  </si>
-  <si>
-    <t>LmtOrderCreationExcel.xlsx</t>
-  </si>
-  <si>
-    <t>PO_NUMBER</t>
-  </si>
-  <si>
-    <t>0000000135</t>
-  </si>
-  <si>
-    <t>Product Exclusion Policy</t>
-  </si>
-  <si>
-    <t>PRODUCT_POLICY</t>
-  </si>
-  <si>
-    <t>PEP</t>
-  </si>
-  <si>
-    <t>ProductExclusionFile.xlsx</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>ProductExclusionFile1.xlsx</t>
-  </si>
-  <si>
-    <t>00Access2024-RQBTESTING</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>Distributor shuffling upload</t>
-  </si>
-  <si>
-    <t>DISTRIBUTOR_SHUFFLING_UPLOAD</t>
-  </si>
-  <si>
-    <t>DistributorShuffling1.xlsx</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>UPLOAD_ONLY</t>
-  </si>
-  <si>
-    <t>DistributorShuffling2.xlsx</t>
-  </si>
-  <si>
-    <t>Distributor Shuffling Upload</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>User Bulk Upload</t>
-  </si>
-  <si>
-    <t>USER_BULK_UPLOAD</t>
-  </si>
-  <si>
-    <t>UserBulkUpload.xlsx</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>Selling Category Bulk Upload</t>
-  </si>
-  <si>
-    <t>SELLING_CATEGORY_BULK_UPLOAD</t>
-  </si>
-  <si>
-    <t>Selling_Category_Bulk_Upload.xlsx</t>
-  </si>
-  <si>
-    <t>leopardPOB - leopardPOB</t>
-  </si>
-  <si>
-    <t>RQBTESTING</t>
-  </si>
-  <si>
-    <t>DEWANHAT</t>
-  </si>
-  <si>
-    <t>DISTRIBUTOR</t>
-  </si>
-  <si>
-    <t>Code*</t>
-  </si>
-  <si>
-    <t>User_</t>
-  </si>
-  <si>
-    <t>Name*</t>
-  </si>
-  <si>
-    <t>Auto_</t>
-  </si>
-  <si>
-    <t>NIC</t>
-  </si>
-  <si>
-    <t>validateMode</t>
-  </si>
-  <si>
-    <t>menuSearch</t>
-  </si>
-  <si>
-    <t>validateScreenId</t>
-  </si>
-  <si>
-    <t>validateGeneratedCol</t>
-  </si>
-  <si>
-    <t>columnId</t>
-  </si>
-  <si>
-    <t>UI_Search</t>
-  </si>
-  <si>
-    <t>dsr profile hq</t>
-  </si>
-  <si>
-    <t>DYL_202044</t>
-  </si>
-  <si>
-    <t>rowfilter_TXT__EPP2DESC</t>
-  </si>
-  <si>
-    <t>product Enrichment Approval</t>
-  </si>
-  <si>
-    <t>Outlet profile HQ</t>
-  </si>
-  <si>
-    <t>DYL_BG1013</t>
-  </si>
-  <si>
-    <t>rowfilter_TXT__EPP1DESC</t>
-  </si>
-  <si>
-    <t>Section Creation HQ</t>
-  </si>
-  <si>
-    <t>DYL_202046</t>
-  </si>
-  <si>
-    <t>Section Code</t>
-  </si>
-  <si>
-    <t>rowfilter_TXT__ENTITYCODE</t>
-  </si>
-  <si>
-    <t>Distributor Profile HQ</t>
-  </si>
-  <si>
-    <t>DYL_L__BusinessEntityProfile</t>
-  </si>
-  <si>
-    <t>Distributor Name*</t>
-  </si>
-  <si>
-    <t>Vehicle Profile</t>
-  </si>
-  <si>
-    <t>DYL_1032</t>
-  </si>
-  <si>
-    <t>Description*</t>
-  </si>
-  <si>
-    <t>rowfilter_Description</t>
-  </si>
-  <si>
-    <t>Price Master Approval</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>bulk order upload</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>User profile</t>
-  </si>
-  <si>
-    <t>0201</t>
-  </si>
-  <si>
-    <t>rowfilter_code</t>
-  </si>
-  <si>
-    <t>SECTION</t>
-  </si>
-  <si>
-    <t>AUTOSEC</t>
-  </si>
-  <si>
-    <t>Key</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>PriceToValidate</t>
-  </si>
-  <si>
-    <t>priceScreenID</t>
-  </si>
-  <si>
-    <t>tradePriceCTN</t>
-  </si>
-  <si>
-    <t>PROD_PRICE</t>
-  </si>
-  <si>
-    <t>ScreenName</t>
-  </si>
-  <si>
-    <t>ScreenId</t>
-  </si>
-  <si>
-    <t>PURCHASE PRICE</t>
-  </si>
-  <si>
-    <t>PURCHASE_PRICE</t>
-  </si>
-  <si>
-    <t>Product Code</t>
-  </si>
-  <si>
-    <t>65150683</t>
+    <t>Distributor Code*,Selling Category Code*</t>
+  </si>
+  <si>
+    <t>Outlet Code*,Outlet Long Name*</t>
   </si>
 </sst>
 </file>
@@ -761,7 +885,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -819,6 +943,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1099,70 +1229,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.1796875" customWidth="1"/>
     <col min="5" max="5" width="25.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="E1" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="F1" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="G1" s="21" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="E2" s="22" t="s">
         <v>156</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>157</v>
       </c>
       <c r="F2" s="22" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="22" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="58" x14ac:dyDescent="0.35">
-      <c r="A3" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>159</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1172,123 +1302,135 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
+      <c r="D4" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>190</v>
+      </c>
       <c r="F4" s="22"/>
       <c r="G4" s="22"/>
     </row>
-    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>160</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="F5" s="22" t="s">
         <v>51</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>44</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D6" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>160</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="F6" s="22" t="s">
         <v>51</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>62</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D7" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="F7" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="G7" s="22" t="s">
         <v>165</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="22"/>
+      <c r="C8" s="22" t="s">
+        <v>209</v>
+      </c>
       <c r="D8" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="E8" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="F8" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="F8" s="22" t="s">
-        <v>169</v>
-      </c>
       <c r="G8" s="22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
+      <c r="C9" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>223</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>224</v>
+      </c>
       <c r="F9" s="22"/>
       <c r="G9" s="22"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>70</v>
@@ -1301,33 +1443,33 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D11" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="E11" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="F11" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="G11" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
@@ -1337,10 +1479,10 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
@@ -1350,10 +1492,10 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
@@ -1363,10 +1505,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>176</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
@@ -1376,7 +1518,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>28</v>
@@ -1389,33 +1531,33 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D17" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="E17" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="F17" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="G17" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>125</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>126</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
@@ -1425,10 +1567,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="19"/>
@@ -1438,39 +1580,56 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B20" s="12" t="s">
-        <v>134</v>
-      </c>
       <c r="C20" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D20" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="F20" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="G20" s="11" t="s">
         <v>179</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="12" t="s">
         <v>137</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>138</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="19"/>
       <c r="E21" s="19"/>
       <c r="F21" s="19"/>
       <c r="G21" s="19"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="B22" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25" t="s">
+        <v>204</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>203</v>
+      </c>
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1479,7 +1638,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="31.54296875" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -1493,7 +1652,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -1511,12 +1670,12 @@
         <v>55</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="6" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>4</v>
@@ -1525,65 +1684,65 @@
         <v>5</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>57</v>
       </c>
       <c r="F2" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="7" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F3" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>33</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>58</v>
       </c>
       <c r="F4" s="29" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="6" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>49</v>
@@ -1592,21 +1751,21 @@
         <v>50</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>59</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>44</v>
@@ -1615,21 +1774,21 @@
         <v>45</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>60</v>
       </c>
       <c r="F6" s="29" t="s">
-        <v>185</v>
+        <v>75</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>155</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>62</v>
@@ -1638,21 +1797,21 @@
         <v>61</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>63</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>64</v>
@@ -1661,19 +1820,21 @@
         <v>65</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>66</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="G8" s="12"/>
+        <v>230</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="9" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>67</v>
@@ -1682,19 +1843,21 @@
         <v>68</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>69</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="G9" s="12"/>
+        <v>230</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="10" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>70</v>
@@ -1703,42 +1866,44 @@
         <v>71</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>72</v>
+        <v>234</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="G10" s="12"/>
+        <v>230</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="C11" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>230</v>
+      </c>
+      <c r="G11" s="11" t="s">
         <v>112</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="6" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>28</v>
@@ -1751,139 +1916,167 @@
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G12" s="12"/>
     </row>
     <row r="13" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B13" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="E13" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>120</v>
-      </c>
       <c r="F13" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G13" s="12"/>
     </row>
     <row r="14" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>123</v>
-      </c>
       <c r="F14" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G14" s="12"/>
     </row>
     <row r="15" spans="1:8" s="19" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="C15" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="D15" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="D15" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>128</v>
-      </c>
       <c r="F15" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="30"/>
     </row>
     <row r="16" spans="1:8" s="19" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="E16" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E16" s="11" t="s">
-        <v>131</v>
-      </c>
       <c r="F16" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G16" s="12"/>
       <c r="H16" s="30"/>
     </row>
     <row r="17" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="D17" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D17" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>136</v>
-      </c>
       <c r="F17" s="29" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="D18" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="F18" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="G18" s="12"/>
+      <c r="G18" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="F19" s="29" t="s">
+        <v>230</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E20" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1893,7 +2086,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="19" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="36.90625" bestFit="1" customWidth="1"/>
@@ -1903,7 +2096,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1917,77 +2110,77 @@
     </row>
     <row r="2" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>28</v>
@@ -1997,12 +2190,12 @@
       </c>
       <c r="D7" s="4" t="str">
         <f ca="1" xml:space="preserve"> TEXT(TODAY() - 4, "yyyy-mm-dd")</f>
-        <v>2026-06-25</v>
+        <v>2026-07-02</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>28</v>
@@ -2012,12 +2205,12 @@
       </c>
       <c r="D8" s="5" t="str">
         <f ca="1">TEXT(TODAY()+2, "yyyy-mm-dd")</f>
-        <v>2026-07-01</v>
+        <v>2026-07-08</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>28</v>
@@ -2026,12 +2219,12 @@
         <v>31</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>28</v>
@@ -2040,12 +2233,12 @@
         <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>4</v>
@@ -2054,12 +2247,12 @@
         <v>9</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>44</v>
@@ -2068,12 +2261,12 @@
         <v>46</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>44</v>
@@ -2082,12 +2275,12 @@
         <v>47</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>44</v>
@@ -2096,12 +2289,12 @@
         <v>9</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>44</v>
@@ -2110,12 +2303,12 @@
         <v>34</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>44</v>
@@ -2124,12 +2317,12 @@
         <v>48</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>62</v>
@@ -2138,12 +2331,12 @@
         <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>62</v>
@@ -2152,12 +2345,12 @@
         <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>64</v>
@@ -2166,133 +2359,203 @@
         <v>47</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D20" t="s">
         <v>83</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>47</v>
       </c>
       <c r="D24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>46</v>
       </c>
       <c r="D27" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D28" t="s">
-        <v>144</v>
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2303,7 +2566,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="24.36328125" customWidth="1"/>
@@ -2315,7 +2578,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2335,7 +2598,7 @@
     </row>
     <row r="2" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -2355,7 +2618,7 @@
     </row>
     <row r="3" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
@@ -2375,7 +2638,7 @@
     </row>
     <row r="4" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
@@ -2393,7 +2656,7 @@
     </row>
     <row r="5" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
@@ -2413,13 +2676,13 @@
     </row>
     <row r="6" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>39</v>
@@ -2431,10 +2694,10 @@
     </row>
     <row r="7" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>35</v>
@@ -2448,10 +2711,10 @@
     </row>
     <row r="8" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>36</v>
@@ -2465,10 +2728,10 @@
     </row>
     <row r="9" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>37</v>
@@ -2482,10 +2745,10 @@
     </row>
     <row r="10" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>38</v>
@@ -2499,10 +2762,10 @@
     </row>
     <row r="11" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>40</v>
@@ -2513,7 +2776,7 @@
     </row>
     <row r="12" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>49</v>
@@ -2533,7 +2796,7 @@
     </row>
     <row r="13" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>49</v>
@@ -2550,7 +2813,7 @@
     </row>
     <row r="14" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>49</v>
@@ -2567,13 +2830,13 @@
     </row>
     <row r="15" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>20</v>
@@ -2584,13 +2847,13 @@
     </row>
     <row r="16" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="C16" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>20</v>
@@ -2599,18 +2862,18 @@
         <v>5</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="C17" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>20</v>
@@ -2619,18 +2882,18 @@
         <v>5</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="C18" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>39</v>
@@ -2641,7 +2904,7 @@
     </row>
     <row r="19" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>44</v>
@@ -2661,13 +2924,13 @@
     </row>
     <row r="20" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>20</v>
@@ -2676,27 +2939,45 @@
         <v>4</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>169</v>
+        <v>208</v>
       </c>
       <c r="D21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="2">
+        <v>2</v>
+      </c>
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E22" s="2">
         <v>4</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>86</v>
+      <c r="F22" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2706,77 +2987,253 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="13.7265625" customWidth="1"/>
-    <col min="3" max="3" width="15.81640625" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" customWidth="1"/>
+    <col min="3" max="3" width="36.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>183</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" t="s">
         <v>190</v>
-      </c>
-      <c r="C5" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>101</v>
+        <v>194</v>
       </c>
       <c r="B6" t="s">
         <v>191</v>
       </c>
-      <c r="C6" t="s">
-        <v>193</v>
+      <c r="C6" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C8" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" t="s">
+        <v>210</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" t="s">
+        <v>202</v>
+      </c>
+      <c r="C10" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" t="s">
+        <v>213</v>
+      </c>
+      <c r="C12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" t="s">
+        <v>215</v>
+      </c>
+      <c r="C14" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" t="s">
+        <v>216</v>
+      </c>
+      <c r="C16" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" t="s">
+        <v>191</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" t="s">
+        <v>228</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" t="s">
+        <v>226</v>
+      </c>
+      <c r="C19" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" t="s">
+        <v>231</v>
+      </c>
+      <c r="C21" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" t="s">
+        <v>231</v>
+      </c>
+      <c r="C22" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>